<commit_message>
Add columns to exported Excel file (ICU sheet)
</commit_message>
<xml_diff>
--- a/notebooks/model_export2.xlsx
+++ b/notebooks/model_export2.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:W7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -817,60 +817,70 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Prob_Pre_ICU</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Prob_Post_ICU</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Pre_Distribution</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Pre_Param1</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Pre_Param2</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Pre_Param3</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Distribution</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Param1</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Param2</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Param3</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Post_Distribution</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Post_Param1</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Post_Param2</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Post_Param3</t>
         </is>
@@ -912,46 +922,52 @@
       <c r="I2" s="2" t="n">
         <v>0.0303030303030303</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="n">
+        <v>0.5303030303030303</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>Lognormal_3P</t>
         </is>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="M2" s="3" t="n">
         <v>-1.065916885862443</v>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="N2" s="3" t="n">
         <v>1.630092753950848</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="O2" s="3" t="n">
         <v>0.07294686252141819</v>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Lognormal_3P</t>
         </is>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="Q2" s="3" t="n">
         <v>1.677315593918787</v>
       </c>
-      <c r="P2" s="3" t="n">
+      <c r="R2" s="3" t="n">
         <v>1.254931464251516</v>
       </c>
-      <c r="Q2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>Lognormal_3P</t>
         </is>
       </c>
-      <c r="S2" s="3" t="n">
+      <c r="U2" s="3" t="n">
         <v>1.628562118722197</v>
       </c>
-      <c r="T2" s="3" t="n">
+      <c r="V2" s="3" t="n">
         <v>1.302401893934868</v>
       </c>
-      <c r="U2" s="3" t="n">
+      <c r="W2" s="3" t="n">
         <v>0.721799957516546</v>
       </c>
     </row>
@@ -1061,7 +1077,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="18">
+    <mergeCell ref="W2:W7"/>
     <mergeCell ref="L2:L7"/>
     <mergeCell ref="S2:S7"/>
     <mergeCell ref="O2:O7"/>
@@ -1077,6 +1094,7 @@
     <mergeCell ref="U2:U7"/>
     <mergeCell ref="N2:N7"/>
     <mergeCell ref="K2:K7"/>
+    <mergeCell ref="V2:V7"/>
     <mergeCell ref="P2:P7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>